<commit_message>
Fuera la cédula y tablas más claras
El cliente no necesita la cédula: se quita del alta, de la ficha, del
CSV, de la plantilla de Excel y de la importación. Los usuarios que ya la
tuvieran guardada dejan de mostrarla; una copia antigua que la traiga se
acepta sin ella.

Tablas: filas alternas, cabecera gris y cifras alineadas a la derecha.
Las cabeceras las pinta ahora el script (va en caché), lo que deja sitio
en la página y en la hoja de estilos, que sigue cabiendo en una sola
respuesta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/herramientas/plantilla-usuarios.xlsx
+++ b/herramientas/plantilla-usuarios.xlsx
@@ -52,7 +52,6 @@
     <col min="1" max="1" width="18" style="1" customWidth="1"/>
     <col min="2" max="2" width="10" style="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -69,11 +68,6 @@
       <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Nombre completo</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Cédula</t>
         </is>
       </c>
     </row>
@@ -111,7 +105,7 @@
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Nombre completo y Cédula: opcionales, para saber quién es cada usuario. La cédula no puede repetirse.</t>
+          <t>Nombre completo: opcional, para saber quién es cada usuario.</t>
         </is>
       </c>
     </row>

</xml_diff>